<commit_message>
update course & course review
</commit_message>
<xml_diff>
--- a/doc/templates/Hango_Course_Import_Template.xlsx
+++ b/doc/templates/Hango_Course_Import_Template.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="23040" windowHeight="9707" activeTab="4"/>
+    <workbookView windowWidth="23040" windowHeight="8987" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="README_AND_RULES" sheetId="1" r:id="rId1"/>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="146" uniqueCount="100">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="143" uniqueCount="97">
   <si>
     <t>Hango Course Import Template - Rules</t>
   </si>
@@ -115,9 +115,6 @@
     <t>Thumbnail URL</t>
   </si>
   <si>
-    <t>Status</t>
-  </si>
-  <si>
     <t>Version</t>
   </si>
   <si>
@@ -139,9 +136,6 @@
     <t>https://example.com/thumb.png</t>
   </si>
   <si>
-    <t>PUBLISHED</t>
-  </si>
-  <si>
     <t>v0.1</t>
   </si>
   <si>
@@ -152,9 +146,6 @@
   </si>
   <si>
     <t>This course provides all knowledges about simple past tense</t>
-  </si>
-  <si>
-    <t>DRAFT</t>
   </si>
   <si>
     <t>SECTIONS OVERVIEW</t>
@@ -1766,7 +1757,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:K22"/>
+  <dimension ref="A1:J22"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="21.6666666666667" customWidth="1"/>
@@ -1776,10 +1767,9 @@
     <col min="5" max="5" width="10.7777777777778" customWidth="1"/>
     <col min="6" max="6" width="8.33333333333333" customWidth="1"/>
     <col min="7" max="7" width="31.5555555555556" customWidth="1"/>
-    <col min="8" max="8" width="13.2222222222222" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="22.8" spans="1:11">
+    <row r="1" ht="22.8" spans="1:10">
       <c r="A1" s="18" t="s">
         <v>19</v>
       </c>
@@ -1790,11 +1780,10 @@
       <c r="F1" s="19"/>
       <c r="G1" s="19"/>
       <c r="H1" s="19"/>
-      <c r="I1" s="19"/>
+      <c r="I1" s="7"/>
       <c r="J1" s="7"/>
-      <c r="K1" s="7"/>
-    </row>
-    <row r="2" s="13" customFormat="1" ht="30" customHeight="1" spans="1:11">
+    </row>
+    <row r="2" s="13" customFormat="1" ht="30" customHeight="1" spans="1:10">
       <c r="A2" s="5" t="s">
         <v>20</v>
       </c>
@@ -1819,44 +1808,38 @@
       <c r="H2" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="I2" s="5" t="s">
+      <c r="I2" s="25"/>
+      <c r="J2" s="26"/>
+    </row>
+    <row r="3" spans="1:10">
+      <c r="A3" s="20" t="s">
         <v>28</v>
       </c>
-      <c r="J2" s="25"/>
-      <c r="K2" s="26"/>
-    </row>
-    <row r="3" spans="1:11">
-      <c r="A3" s="20" t="s">
+      <c r="B3" s="20" t="s">
         <v>29</v>
       </c>
-      <c r="B3" s="20" t="s">
+      <c r="C3" s="20" t="s">
         <v>30</v>
       </c>
-      <c r="C3" s="20" t="s">
+      <c r="D3" s="20" t="s">
         <v>31</v>
       </c>
-      <c r="D3" s="20" t="s">
+      <c r="E3" s="21" t="s">
         <v>32</v>
-      </c>
-      <c r="E3" s="21" t="s">
-        <v>33</v>
       </c>
       <c r="F3" s="20">
         <v>0</v>
       </c>
       <c r="G3" s="20" t="s">
+        <v>33</v>
+      </c>
+      <c r="H3" s="20" t="s">
         <v>34</v>
       </c>
-      <c r="H3" s="20" t="s">
-        <v>35</v>
-      </c>
-      <c r="I3" s="20" t="s">
-        <v>36</v>
-      </c>
+      <c r="I3" s="7"/>
       <c r="J3" s="7"/>
-      <c r="K3" s="7"/>
-    </row>
-    <row r="4" spans="1:11">
+    </row>
+    <row r="4" spans="1:10">
       <c r="A4" s="20"/>
       <c r="B4" s="20"/>
       <c r="C4" s="20"/>
@@ -1865,11 +1848,10 @@
       <c r="F4" s="20"/>
       <c r="G4" s="20"/>
       <c r="H4" s="20"/>
-      <c r="I4" s="20"/>
+      <c r="I4" s="7"/>
       <c r="J4" s="7"/>
-      <c r="K4" s="7"/>
-    </row>
-    <row r="5" spans="1:11">
+    </row>
+    <row r="5" spans="1:10">
       <c r="A5" s="20"/>
       <c r="B5" s="20"/>
       <c r="C5" s="20"/>
@@ -1878,11 +1860,10 @@
       <c r="F5" s="20"/>
       <c r="G5" s="20"/>
       <c r="H5" s="20"/>
-      <c r="I5" s="20"/>
+      <c r="I5" s="7"/>
       <c r="J5" s="7"/>
-      <c r="K5" s="7"/>
-    </row>
-    <row r="6" spans="1:11">
+    </row>
+    <row r="6" spans="1:10">
       <c r="A6" s="20"/>
       <c r="B6" s="20"/>
       <c r="C6" s="20"/>
@@ -1891,11 +1872,10 @@
       <c r="F6" s="20"/>
       <c r="G6" s="20"/>
       <c r="H6" s="20"/>
-      <c r="I6" s="20"/>
+      <c r="I6" s="7"/>
       <c r="J6" s="7"/>
-      <c r="K6" s="7"/>
-    </row>
-    <row r="7" spans="1:11">
+    </row>
+    <row r="7" spans="1:10">
       <c r="A7" s="20"/>
       <c r="B7" s="20"/>
       <c r="C7" s="20"/>
@@ -1904,42 +1884,38 @@
       <c r="F7" s="20"/>
       <c r="G7" s="20"/>
       <c r="H7" s="20"/>
-      <c r="I7" s="20"/>
+      <c r="I7" s="7"/>
       <c r="J7" s="7"/>
-      <c r="K7" s="7"/>
-    </row>
-    <row r="8" spans="1:11">
+    </row>
+    <row r="8" spans="1:10">
       <c r="A8" s="20" t="s">
+        <v>35</v>
+      </c>
+      <c r="B8" s="20" t="s">
+        <v>36</v>
+      </c>
+      <c r="C8" s="20" t="s">
         <v>37</v>
       </c>
-      <c r="B8" s="20" t="s">
-        <v>38</v>
-      </c>
-      <c r="C8" s="20" t="s">
-        <v>39</v>
-      </c>
       <c r="D8" s="20" t="s">
+        <v>31</v>
+      </c>
+      <c r="E8" s="21" t="s">
         <v>32</v>
-      </c>
-      <c r="E8" s="21" t="s">
-        <v>33</v>
       </c>
       <c r="F8" s="20">
         <v>0</v>
       </c>
       <c r="G8" s="20" t="s">
+        <v>33</v>
+      </c>
+      <c r="H8" s="20" t="s">
         <v>34</v>
       </c>
-      <c r="H8" s="20" t="s">
-        <v>40</v>
-      </c>
-      <c r="I8" s="20" t="s">
-        <v>36</v>
-      </c>
+      <c r="I8" s="7"/>
       <c r="J8" s="7"/>
-      <c r="K8" s="7"/>
-    </row>
-    <row r="9" spans="1:11">
+    </row>
+    <row r="9" spans="1:10">
       <c r="A9" s="20"/>
       <c r="B9" s="20"/>
       <c r="C9" s="20"/>
@@ -1948,11 +1924,10 @@
       <c r="F9" s="20"/>
       <c r="G9" s="20"/>
       <c r="H9" s="20"/>
-      <c r="I9" s="20"/>
+      <c r="I9" s="7"/>
       <c r="J9" s="7"/>
-      <c r="K9" s="7"/>
-    </row>
-    <row r="10" spans="1:11">
+    </row>
+    <row r="10" spans="1:10">
       <c r="A10" s="20"/>
       <c r="B10" s="20"/>
       <c r="C10" s="20"/>
@@ -1961,11 +1936,10 @@
       <c r="F10" s="20"/>
       <c r="G10" s="20"/>
       <c r="H10" s="20"/>
-      <c r="I10" s="20"/>
+      <c r="I10" s="7"/>
       <c r="J10" s="7"/>
-      <c r="K10" s="7"/>
-    </row>
-    <row r="11" spans="1:11">
+    </row>
+    <row r="11" spans="1:10">
       <c r="A11" s="20"/>
       <c r="B11" s="20"/>
       <c r="C11" s="20"/>
@@ -1974,11 +1948,10 @@
       <c r="F11" s="20"/>
       <c r="G11" s="20"/>
       <c r="H11" s="20"/>
-      <c r="I11" s="20"/>
+      <c r="I11" s="7"/>
       <c r="J11" s="7"/>
-      <c r="K11" s="7"/>
-    </row>
-    <row r="12" spans="1:11">
+    </row>
+    <row r="12" spans="1:10">
       <c r="A12" s="20"/>
       <c r="B12" s="20"/>
       <c r="C12" s="20"/>
@@ -1987,11 +1960,10 @@
       <c r="F12" s="20"/>
       <c r="G12" s="20"/>
       <c r="H12" s="20"/>
-      <c r="I12" s="20"/>
+      <c r="I12" s="7"/>
       <c r="J12" s="7"/>
-      <c r="K12" s="7"/>
-    </row>
-    <row r="13" spans="1:11">
+    </row>
+    <row r="13" spans="1:10">
       <c r="A13" s="20"/>
       <c r="B13" s="20"/>
       <c r="C13" s="20"/>
@@ -2000,11 +1972,10 @@
       <c r="F13" s="20"/>
       <c r="G13" s="20"/>
       <c r="H13" s="20"/>
-      <c r="I13" s="20"/>
+      <c r="I13" s="7"/>
       <c r="J13" s="7"/>
-      <c r="K13" s="7"/>
-    </row>
-    <row r="14" spans="1:11">
+    </row>
+    <row r="14" spans="1:10">
       <c r="A14" s="20"/>
       <c r="B14" s="20"/>
       <c r="C14" s="20"/>
@@ -2013,11 +1984,10 @@
       <c r="F14" s="20"/>
       <c r="G14" s="20"/>
       <c r="H14" s="20"/>
-      <c r="I14" s="20"/>
+      <c r="I14" s="7"/>
       <c r="J14" s="7"/>
-      <c r="K14" s="7"/>
-    </row>
-    <row r="15" spans="1:11">
+    </row>
+    <row r="15" spans="1:10">
       <c r="A15" s="20"/>
       <c r="B15" s="20"/>
       <c r="C15" s="20"/>
@@ -2026,11 +1996,10 @@
       <c r="F15" s="20"/>
       <c r="G15" s="20"/>
       <c r="H15" s="20"/>
-      <c r="I15" s="20"/>
+      <c r="I15" s="7"/>
       <c r="J15" s="7"/>
-      <c r="K15" s="7"/>
-    </row>
-    <row r="16" ht="12" customHeight="1" spans="1:11">
+    </row>
+    <row r="16" ht="12" customHeight="1" spans="1:10">
       <c r="A16" s="20"/>
       <c r="B16" s="20"/>
       <c r="C16" s="20"/>
@@ -2039,11 +2008,10 @@
       <c r="F16" s="20"/>
       <c r="G16" s="20"/>
       <c r="H16" s="20"/>
-      <c r="I16" s="20"/>
+      <c r="I16" s="7"/>
       <c r="J16" s="7"/>
-      <c r="K16" s="7"/>
-    </row>
-    <row r="17" spans="1:11">
+    </row>
+    <row r="17" spans="1:10">
       <c r="A17" s="20"/>
       <c r="B17" s="20"/>
       <c r="C17" s="20"/>
@@ -2052,11 +2020,10 @@
       <c r="F17" s="20"/>
       <c r="G17" s="20"/>
       <c r="H17" s="20"/>
-      <c r="I17" s="20"/>
+      <c r="I17" s="7"/>
       <c r="J17" s="7"/>
-      <c r="K17" s="7"/>
-    </row>
-    <row r="18" spans="1:11">
+    </row>
+    <row r="18" spans="1:10">
       <c r="A18" s="20"/>
       <c r="B18" s="20"/>
       <c r="C18" s="20"/>
@@ -2065,11 +2032,10 @@
       <c r="F18" s="20"/>
       <c r="G18" s="20"/>
       <c r="H18" s="20"/>
-      <c r="I18" s="20"/>
+      <c r="I18" s="7"/>
       <c r="J18" s="7"/>
-      <c r="K18" s="7"/>
-    </row>
-    <row r="19" spans="1:11">
+    </row>
+    <row r="19" spans="1:10">
       <c r="A19" s="20"/>
       <c r="B19" s="20"/>
       <c r="C19" s="20"/>
@@ -2078,11 +2044,10 @@
       <c r="F19" s="20"/>
       <c r="G19" s="20"/>
       <c r="H19" s="20"/>
-      <c r="I19" s="20"/>
+      <c r="I19" s="7"/>
       <c r="J19" s="7"/>
-      <c r="K19" s="7"/>
-    </row>
-    <row r="20" spans="1:11">
+    </row>
+    <row r="20" spans="1:10">
       <c r="A20" s="20"/>
       <c r="B20" s="20"/>
       <c r="C20" s="20"/>
@@ -2091,11 +2056,10 @@
       <c r="F20" s="20"/>
       <c r="G20" s="20"/>
       <c r="H20" s="20"/>
-      <c r="I20" s="20"/>
+      <c r="I20" s="7"/>
       <c r="J20" s="7"/>
-      <c r="K20" s="7"/>
-    </row>
-    <row r="21" spans="1:11">
+    </row>
+    <row r="21" spans="1:10">
       <c r="A21" s="20"/>
       <c r="B21" s="20"/>
       <c r="C21" s="20"/>
@@ -2104,11 +2068,10 @@
       <c r="F21" s="20"/>
       <c r="G21" s="20"/>
       <c r="H21" s="20"/>
-      <c r="I21" s="20"/>
+      <c r="I21" s="7"/>
       <c r="J21" s="7"/>
-      <c r="K21" s="7"/>
-    </row>
-    <row r="22" spans="1:11">
+    </row>
+    <row r="22" spans="1:10">
       <c r="A22" s="20"/>
       <c r="B22" s="20"/>
       <c r="C22" s="20"/>
@@ -2117,13 +2080,12 @@
       <c r="F22" s="20"/>
       <c r="G22" s="20"/>
       <c r="H22" s="20"/>
-      <c r="I22" s="20"/>
+      <c r="I22" s="7"/>
       <c r="J22" s="7"/>
-      <c r="K22" s="7"/>
     </row>
   </sheetData>
-  <mergeCells count="37">
-    <mergeCell ref="A1:I1"/>
+  <mergeCells count="33">
+    <mergeCell ref="A1:H1"/>
     <mergeCell ref="A3:A7"/>
     <mergeCell ref="A8:A12"/>
     <mergeCell ref="A13:A17"/>
@@ -2156,17 +2118,10 @@
     <mergeCell ref="H8:H12"/>
     <mergeCell ref="H13:H17"/>
     <mergeCell ref="H18:H22"/>
-    <mergeCell ref="I3:I7"/>
-    <mergeCell ref="I8:I12"/>
-    <mergeCell ref="I13:I17"/>
-    <mergeCell ref="I18:I22"/>
   </mergeCells>
-  <dataValidations count="2">
+  <dataValidations count="1">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E3:E22">
       <formula1>"BEGINNER,INTERMEDIATE,ADVANCE"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H3:H12">
-      <formula1>"PUBLISHED,DRAFT,PRIVATE"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2191,7 +2146,7 @@
   <sheetData>
     <row r="1" ht="20" customHeight="1" spans="1:6">
       <c r="A1" s="15" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="B1" s="15"/>
       <c r="C1" s="15"/>
@@ -2204,59 +2159,59 @@
         <v>20</v>
       </c>
       <c r="B2" s="16" t="s">
+        <v>39</v>
+      </c>
+      <c r="C2" s="16" t="s">
+        <v>40</v>
+      </c>
+      <c r="D2" s="16" t="s">
+        <v>41</v>
+      </c>
+      <c r="E2" s="16" t="s">
         <v>42</v>
       </c>
-      <c r="C2" s="16" t="s">
-        <v>43</v>
-      </c>
-      <c r="D2" s="16" t="s">
-        <v>44</v>
-      </c>
-      <c r="E2" s="16" t="s">
-        <v>45</v>
-      </c>
       <c r="F2" s="16" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="3" ht="20" customHeight="1" spans="1:6">
       <c r="A3" s="9" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B3" s="9" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="C3" s="9" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="D3" s="17" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="E3" s="9">
         <v>1</v>
       </c>
       <c r="F3" s="9" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
     </row>
     <row r="4" ht="20" customHeight="1" spans="1:6">
       <c r="A4" s="9" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="D4" s="17" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="E4" s="9">
         <v>2</v>
       </c>
       <c r="F4" s="9" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
     </row>
     <row r="5" ht="20" customHeight="1"/>
@@ -2320,7 +2275,7 @@
   <sheetData>
     <row r="1" ht="22.8" spans="1:15">
       <c r="A1" s="10" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="B1" s="11"/>
       <c r="C1" s="11"/>
@@ -2342,125 +2297,125 @@
         <v>20</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="C2" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="D2" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="E2" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="F2" s="5" t="s">
         <v>52</v>
       </c>
-      <c r="D2" s="5" t="s">
+      <c r="G2" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="E2" s="5" t="s">
+      <c r="H2" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="F2" s="5" t="s">
+      <c r="I2" s="5" t="s">
         <v>55</v>
       </c>
-      <c r="G2" s="5" t="s">
+      <c r="J2" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="H2" s="5" t="s">
+      <c r="K2" s="5" t="s">
         <v>57</v>
       </c>
-      <c r="I2" s="5" t="s">
+      <c r="L2" s="5" t="s">
         <v>58</v>
       </c>
-      <c r="J2" s="5" t="s">
+      <c r="M2" s="5" t="s">
         <v>59</v>
       </c>
-      <c r="K2" s="5" t="s">
+      <c r="N2" s="5" t="s">
         <v>60</v>
       </c>
-      <c r="L2" s="5" t="s">
-        <v>61</v>
-      </c>
-      <c r="M2" s="5" t="s">
-        <v>62</v>
-      </c>
-      <c r="N2" s="5" t="s">
-        <v>63</v>
-      </c>
       <c r="O2" s="5" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="3" ht="20" customHeight="1" spans="1:15">
       <c r="A3" s="12" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B3" s="12" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="C3" s="12" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="D3" s="12" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="E3" s="12">
         <v>1</v>
       </c>
       <c r="F3" s="12" t="s">
+        <v>63</v>
+      </c>
+      <c r="G3" s="12" t="s">
+        <v>64</v>
+      </c>
+      <c r="H3" s="12" t="s">
+        <v>65</v>
+      </c>
+      <c r="I3" s="12" t="s">
+        <v>65</v>
+      </c>
+      <c r="J3" s="12" t="s">
+        <v>65</v>
+      </c>
+      <c r="K3" s="12" t="s">
+        <v>65</v>
+      </c>
+      <c r="L3" s="12" t="s">
+        <v>65</v>
+      </c>
+      <c r="M3" s="12" t="s">
         <v>66</v>
-      </c>
-      <c r="G3" s="12" t="s">
-        <v>67</v>
-      </c>
-      <c r="H3" s="12" t="s">
-        <v>68</v>
-      </c>
-      <c r="I3" s="12" t="s">
-        <v>68</v>
-      </c>
-      <c r="J3" s="12" t="s">
-        <v>68</v>
-      </c>
-      <c r="K3" s="12" t="s">
-        <v>68</v>
-      </c>
-      <c r="L3" s="12" t="s">
-        <v>68</v>
-      </c>
-      <c r="M3" s="12" t="s">
-        <v>69</v>
       </c>
       <c r="N3" s="12">
         <v>10</v>
       </c>
       <c r="O3" s="12" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
     </row>
     <row r="4" ht="20" customHeight="1" spans="1:15">
       <c r="A4" s="12" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B4" s="12" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="C4" s="12" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="D4" s="12" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="E4" s="12">
         <v>2</v>
       </c>
       <c r="F4" s="12" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="G4" s="12" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="H4" s="12" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="I4" s="12" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="J4" s="12" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="K4" s="12">
         <v>360</v>
@@ -2469,60 +2424,60 @@
         <v>104857600</v>
       </c>
       <c r="M4" s="12" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="N4" s="12">
         <v>15</v>
       </c>
       <c r="O4" s="12" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
     </row>
     <row r="5" ht="20" customHeight="1" spans="1:15">
       <c r="A5" s="12" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B5" s="12" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="C5" s="12" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="D5" s="12" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="E5" s="12">
         <v>1</v>
       </c>
       <c r="F5" s="12" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="G5" s="12" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="H5" s="12" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="I5" s="12" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="J5" s="12" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="K5" s="12" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="L5" s="12" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="M5" s="12" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="N5" s="12">
         <v>20</v>
       </c>
       <c r="O5" s="12" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1" spans="1:15">
@@ -2746,7 +2701,7 @@
     <row r="1" ht="23.4" spans="4:16">
       <c r="D1" s="4"/>
       <c r="E1" s="4" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="F1" s="4"/>
       <c r="G1" s="4"/>
@@ -2765,43 +2720,43 @@
         <v>20</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="D2" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="E2" s="6" t="s">
+        <v>79</v>
+      </c>
+      <c r="F2" s="6" t="s">
+        <v>80</v>
+      </c>
+      <c r="G2" s="6" t="s">
         <v>81</v>
       </c>
-      <c r="E2" s="6" t="s">
+      <c r="H2" s="6" t="s">
         <v>82</v>
       </c>
-      <c r="F2" s="6" t="s">
+      <c r="I2" s="6" t="s">
         <v>83</v>
       </c>
-      <c r="G2" s="6" t="s">
+      <c r="J2" s="6" t="s">
         <v>84</v>
       </c>
-      <c r="H2" s="6" t="s">
+      <c r="K2" s="6" t="s">
         <v>85</v>
       </c>
-      <c r="I2" s="6" t="s">
+      <c r="L2" s="6" t="s">
         <v>86</v>
       </c>
-      <c r="J2" s="6" t="s">
+      <c r="M2" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="N2" s="6" t="s">
         <v>87</v>
-      </c>
-      <c r="K2" s="6" t="s">
-        <v>88</v>
-      </c>
-      <c r="L2" s="6" t="s">
-        <v>89</v>
-      </c>
-      <c r="M2" s="6" t="s">
-        <v>54</v>
-      </c>
-      <c r="N2" s="6" t="s">
-        <v>90</v>
       </c>
       <c r="O2" s="6" t="s">
         <v>24</v>
@@ -2857,7 +2812,7 @@
   <sheetData>
     <row r="1" s="1" customFormat="1" ht="30" customHeight="1" spans="1:2">
       <c r="A1" s="2" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>22</v>
@@ -2868,47 +2823,47 @@
         <v>20</v>
       </c>
       <c r="B2" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
     </row>
     <row r="3" ht="20" customHeight="1" spans="1:2">
       <c r="A3" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="B3" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
     </row>
     <row r="4" ht="20" customHeight="1" spans="1:2">
       <c r="A4" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="B4" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
     </row>
     <row r="5" ht="20" customHeight="1" spans="1:2">
       <c r="A5" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="B5" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1" spans="1:2">
       <c r="A6" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="B6" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
     </row>
     <row r="7" ht="20" customHeight="1" spans="1:2">
       <c r="A7" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="B7" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
update course version trainer & learner
</commit_message>
<xml_diff>
--- a/doc/templates/Hango_Course_Import_Template.xlsx
+++ b/doc/templates/Hango_Course_Import_Template.xlsx
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="143" uniqueCount="97">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="133" uniqueCount="95">
   <si>
     <t>Hango Course Import Template - Rules</t>
   </si>
@@ -115,9 +115,6 @@
     <t>Thumbnail URL</t>
   </si>
   <si>
-    <t>Version</t>
-  </si>
-  <si>
     <t>COURSE_001</t>
   </si>
   <si>
@@ -134,9 +131,6 @@
   </si>
   <si>
     <t>https://example.com/thumb.png</t>
-  </si>
-  <si>
-    <t>v0.1</t>
   </si>
   <si>
     <t>COURSE_002</t>
@@ -1163,6 +1157,9 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
@@ -1177,9 +1174,6 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1757,7 +1751,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:J22"/>
+  <dimension ref="A1:I22"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="21.6666666666667" customWidth="1"/>
@@ -1769,7 +1763,7 @@
     <col min="7" max="7" width="31.5555555555556" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="22.8" spans="1:10">
+    <row r="1" ht="22.8" spans="1:9">
       <c r="A1" s="18" t="s">
         <v>19</v>
       </c>
@@ -1779,11 +1773,10 @@
       <c r="E1" s="19"/>
       <c r="F1" s="19"/>
       <c r="G1" s="19"/>
-      <c r="H1" s="19"/>
+      <c r="H1" s="7"/>
       <c r="I1" s="7"/>
-      <c r="J1" s="7"/>
-    </row>
-    <row r="2" s="13" customFormat="1" ht="30" customHeight="1" spans="1:10">
+    </row>
+    <row r="2" s="13" customFormat="1" ht="30" customHeight="1" spans="1:9">
       <c r="A2" s="5" t="s">
         <v>20</v>
       </c>
@@ -1805,287 +1798,260 @@
       <c r="G2" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="H2" s="5" t="s">
+      <c r="H2" s="20"/>
+      <c r="I2" s="26"/>
+    </row>
+    <row r="3" spans="1:9">
+      <c r="A3" s="21" t="s">
         <v>27</v>
       </c>
-      <c r="I2" s="25"/>
-      <c r="J2" s="26"/>
-    </row>
-    <row r="3" spans="1:10">
-      <c r="A3" s="20" t="s">
+      <c r="B3" s="21" t="s">
         <v>28</v>
       </c>
-      <c r="B3" s="20" t="s">
+      <c r="C3" s="21" t="s">
         <v>29</v>
       </c>
-      <c r="C3" s="20" t="s">
+      <c r="D3" s="21" t="s">
         <v>30</v>
       </c>
-      <c r="D3" s="20" t="s">
+      <c r="E3" s="22" t="s">
         <v>31</v>
       </c>
-      <c r="E3" s="21" t="s">
+      <c r="F3" s="21">
+        <v>0</v>
+      </c>
+      <c r="G3" s="21" t="s">
         <v>32</v>
       </c>
-      <c r="F3" s="20">
+      <c r="H3" s="7"/>
+      <c r="I3" s="7"/>
+    </row>
+    <row r="4" spans="1:9">
+      <c r="A4" s="21"/>
+      <c r="B4" s="21"/>
+      <c r="C4" s="21"/>
+      <c r="D4" s="21"/>
+      <c r="E4" s="22"/>
+      <c r="F4" s="21"/>
+      <c r="G4" s="21"/>
+      <c r="H4" s="7"/>
+      <c r="I4" s="7"/>
+    </row>
+    <row r="5" spans="1:9">
+      <c r="A5" s="21"/>
+      <c r="B5" s="21"/>
+      <c r="C5" s="21"/>
+      <c r="D5" s="21"/>
+      <c r="E5" s="22"/>
+      <c r="F5" s="21"/>
+      <c r="G5" s="21"/>
+      <c r="H5" s="7"/>
+      <c r="I5" s="7"/>
+    </row>
+    <row r="6" spans="1:9">
+      <c r="A6" s="21"/>
+      <c r="B6" s="21"/>
+      <c r="C6" s="21"/>
+      <c r="D6" s="21"/>
+      <c r="E6" s="22"/>
+      <c r="F6" s="21"/>
+      <c r="G6" s="21"/>
+      <c r="H6" s="7"/>
+      <c r="I6" s="7"/>
+    </row>
+    <row r="7" spans="1:9">
+      <c r="A7" s="21"/>
+      <c r="B7" s="21"/>
+      <c r="C7" s="21"/>
+      <c r="D7" s="21"/>
+      <c r="E7" s="22"/>
+      <c r="F7" s="21"/>
+      <c r="G7" s="21"/>
+      <c r="H7" s="7"/>
+      <c r="I7" s="7"/>
+    </row>
+    <row r="8" spans="1:9">
+      <c r="A8" s="21" t="s">
+        <v>33</v>
+      </c>
+      <c r="B8" s="21" t="s">
+        <v>34</v>
+      </c>
+      <c r="C8" s="21" t="s">
+        <v>35</v>
+      </c>
+      <c r="D8" s="21" t="s">
+        <v>30</v>
+      </c>
+      <c r="E8" s="22" t="s">
+        <v>31</v>
+      </c>
+      <c r="F8" s="21">
         <v>0</v>
       </c>
-      <c r="G3" s="20" t="s">
-        <v>33</v>
-      </c>
-      <c r="H3" s="20" t="s">
-        <v>34</v>
-      </c>
-      <c r="I3" s="7"/>
-      <c r="J3" s="7"/>
-    </row>
-    <row r="4" spans="1:10">
-      <c r="A4" s="20"/>
-      <c r="B4" s="20"/>
-      <c r="C4" s="20"/>
-      <c r="D4" s="20"/>
-      <c r="E4" s="21"/>
-      <c r="F4" s="20"/>
-      <c r="G4" s="20"/>
-      <c r="H4" s="20"/>
-      <c r="I4" s="7"/>
-      <c r="J4" s="7"/>
-    </row>
-    <row r="5" spans="1:10">
-      <c r="A5" s="20"/>
-      <c r="B5" s="20"/>
-      <c r="C5" s="20"/>
-      <c r="D5" s="20"/>
-      <c r="E5" s="21"/>
-      <c r="F5" s="20"/>
-      <c r="G5" s="20"/>
-      <c r="H5" s="20"/>
-      <c r="I5" s="7"/>
-      <c r="J5" s="7"/>
-    </row>
-    <row r="6" spans="1:10">
-      <c r="A6" s="20"/>
-      <c r="B6" s="20"/>
-      <c r="C6" s="20"/>
-      <c r="D6" s="20"/>
-      <c r="E6" s="21"/>
-      <c r="F6" s="20"/>
-      <c r="G6" s="20"/>
-      <c r="H6" s="20"/>
-      <c r="I6" s="7"/>
-      <c r="J6" s="7"/>
-    </row>
-    <row r="7" spans="1:10">
-      <c r="A7" s="20"/>
-      <c r="B7" s="20"/>
-      <c r="C7" s="20"/>
-      <c r="D7" s="20"/>
-      <c r="E7" s="21"/>
-      <c r="F7" s="20"/>
-      <c r="G7" s="20"/>
-      <c r="H7" s="20"/>
-      <c r="I7" s="7"/>
-      <c r="J7" s="7"/>
-    </row>
-    <row r="8" spans="1:10">
-      <c r="A8" s="20" t="s">
-        <v>35</v>
-      </c>
-      <c r="B8" s="20" t="s">
-        <v>36</v>
-      </c>
-      <c r="C8" s="20" t="s">
-        <v>37</v>
-      </c>
-      <c r="D8" s="20" t="s">
-        <v>31</v>
-      </c>
-      <c r="E8" s="21" t="s">
+      <c r="G8" s="21" t="s">
         <v>32</v>
       </c>
-      <c r="F8" s="20">
-        <v>0</v>
-      </c>
-      <c r="G8" s="20" t="s">
-        <v>33</v>
-      </c>
-      <c r="H8" s="20" t="s">
-        <v>34</v>
-      </c>
+      <c r="H8" s="7"/>
       <c r="I8" s="7"/>
-      <c r="J8" s="7"/>
-    </row>
-    <row r="9" spans="1:10">
-      <c r="A9" s="20"/>
-      <c r="B9" s="20"/>
-      <c r="C9" s="20"/>
-      <c r="D9" s="20"/>
-      <c r="E9" s="21"/>
-      <c r="F9" s="20"/>
-      <c r="G9" s="20"/>
-      <c r="H9" s="20"/>
+    </row>
+    <row r="9" spans="1:9">
+      <c r="A9" s="21"/>
+      <c r="B9" s="21"/>
+      <c r="C9" s="21"/>
+      <c r="D9" s="21"/>
+      <c r="E9" s="22"/>
+      <c r="F9" s="21"/>
+      <c r="G9" s="21"/>
+      <c r="H9" s="7"/>
       <c r="I9" s="7"/>
-      <c r="J9" s="7"/>
-    </row>
-    <row r="10" spans="1:10">
-      <c r="A10" s="20"/>
-      <c r="B10" s="20"/>
-      <c r="C10" s="20"/>
-      <c r="D10" s="20"/>
-      <c r="E10" s="21"/>
-      <c r="F10" s="20"/>
-      <c r="G10" s="20"/>
-      <c r="H10" s="20"/>
+    </row>
+    <row r="10" spans="1:9">
+      <c r="A10" s="21"/>
+      <c r="B10" s="21"/>
+      <c r="C10" s="21"/>
+      <c r="D10" s="21"/>
+      <c r="E10" s="22"/>
+      <c r="F10" s="21"/>
+      <c r="G10" s="21"/>
+      <c r="H10" s="7"/>
       <c r="I10" s="7"/>
-      <c r="J10" s="7"/>
-    </row>
-    <row r="11" spans="1:10">
-      <c r="A11" s="20"/>
-      <c r="B11" s="20"/>
-      <c r="C11" s="20"/>
-      <c r="D11" s="20"/>
-      <c r="E11" s="21"/>
-      <c r="F11" s="20"/>
-      <c r="G11" s="20"/>
-      <c r="H11" s="20"/>
+    </row>
+    <row r="11" spans="1:9">
+      <c r="A11" s="21"/>
+      <c r="B11" s="21"/>
+      <c r="C11" s="21"/>
+      <c r="D11" s="21"/>
+      <c r="E11" s="22"/>
+      <c r="F11" s="21"/>
+      <c r="G11" s="21"/>
+      <c r="H11" s="7"/>
       <c r="I11" s="7"/>
-      <c r="J11" s="7"/>
-    </row>
-    <row r="12" spans="1:10">
-      <c r="A12" s="20"/>
-      <c r="B12" s="20"/>
-      <c r="C12" s="20"/>
-      <c r="D12" s="20"/>
-      <c r="E12" s="21"/>
-      <c r="F12" s="20"/>
-      <c r="G12" s="20"/>
-      <c r="H12" s="20"/>
+    </row>
+    <row r="12" spans="1:9">
+      <c r="A12" s="21"/>
+      <c r="B12" s="21"/>
+      <c r="C12" s="21"/>
+      <c r="D12" s="21"/>
+      <c r="E12" s="22"/>
+      <c r="F12" s="21"/>
+      <c r="G12" s="21"/>
+      <c r="H12" s="7"/>
       <c r="I12" s="7"/>
-      <c r="J12" s="7"/>
-    </row>
-    <row r="13" spans="1:10">
-      <c r="A13" s="20"/>
-      <c r="B13" s="20"/>
-      <c r="C13" s="20"/>
-      <c r="D13" s="20"/>
-      <c r="E13" s="22"/>
-      <c r="F13" s="20"/>
-      <c r="G13" s="20"/>
-      <c r="H13" s="20"/>
+    </row>
+    <row r="13" spans="1:9">
+      <c r="A13" s="21"/>
+      <c r="B13" s="21"/>
+      <c r="C13" s="21"/>
+      <c r="D13" s="21"/>
+      <c r="E13" s="23"/>
+      <c r="F13" s="21"/>
+      <c r="G13" s="21"/>
+      <c r="H13" s="7"/>
       <c r="I13" s="7"/>
-      <c r="J13" s="7"/>
-    </row>
-    <row r="14" spans="1:10">
-      <c r="A14" s="20"/>
-      <c r="B14" s="20"/>
-      <c r="C14" s="20"/>
-      <c r="D14" s="20"/>
-      <c r="E14" s="23"/>
-      <c r="F14" s="20"/>
-      <c r="G14" s="20"/>
-      <c r="H14" s="20"/>
+    </row>
+    <row r="14" spans="1:9">
+      <c r="A14" s="21"/>
+      <c r="B14" s="21"/>
+      <c r="C14" s="21"/>
+      <c r="D14" s="21"/>
+      <c r="E14" s="24"/>
+      <c r="F14" s="21"/>
+      <c r="G14" s="21"/>
+      <c r="H14" s="7"/>
       <c r="I14" s="7"/>
-      <c r="J14" s="7"/>
-    </row>
-    <row r="15" spans="1:10">
-      <c r="A15" s="20"/>
-      <c r="B15" s="20"/>
-      <c r="C15" s="20"/>
-      <c r="D15" s="20"/>
-      <c r="E15" s="23"/>
-      <c r="F15" s="20"/>
-      <c r="G15" s="20"/>
-      <c r="H15" s="20"/>
+    </row>
+    <row r="15" spans="1:9">
+      <c r="A15" s="21"/>
+      <c r="B15" s="21"/>
+      <c r="C15" s="21"/>
+      <c r="D15" s="21"/>
+      <c r="E15" s="24"/>
+      <c r="F15" s="21"/>
+      <c r="G15" s="21"/>
+      <c r="H15" s="7"/>
       <c r="I15" s="7"/>
-      <c r="J15" s="7"/>
-    </row>
-    <row r="16" ht="12" customHeight="1" spans="1:10">
-      <c r="A16" s="20"/>
-      <c r="B16" s="20"/>
-      <c r="C16" s="20"/>
-      <c r="D16" s="20"/>
-      <c r="E16" s="23"/>
-      <c r="F16" s="20"/>
-      <c r="G16" s="20"/>
-      <c r="H16" s="20"/>
+    </row>
+    <row r="16" ht="12" customHeight="1" spans="1:9">
+      <c r="A16" s="21"/>
+      <c r="B16" s="21"/>
+      <c r="C16" s="21"/>
+      <c r="D16" s="21"/>
+      <c r="E16" s="24"/>
+      <c r="F16" s="21"/>
+      <c r="G16" s="21"/>
+      <c r="H16" s="7"/>
       <c r="I16" s="7"/>
-      <c r="J16" s="7"/>
-    </row>
-    <row r="17" spans="1:10">
-      <c r="A17" s="20"/>
-      <c r="B17" s="20"/>
-      <c r="C17" s="20"/>
-      <c r="D17" s="20"/>
-      <c r="E17" s="24"/>
-      <c r="F17" s="20"/>
-      <c r="G17" s="20"/>
-      <c r="H17" s="20"/>
+    </row>
+    <row r="17" spans="1:9">
+      <c r="A17" s="21"/>
+      <c r="B17" s="21"/>
+      <c r="C17" s="21"/>
+      <c r="D17" s="21"/>
+      <c r="E17" s="25"/>
+      <c r="F17" s="21"/>
+      <c r="G17" s="21"/>
+      <c r="H17" s="7"/>
       <c r="I17" s="7"/>
-      <c r="J17" s="7"/>
-    </row>
-    <row r="18" spans="1:10">
-      <c r="A18" s="20"/>
-      <c r="B18" s="20"/>
-      <c r="C18" s="20"/>
-      <c r="D18" s="20"/>
-      <c r="E18" s="22"/>
-      <c r="F18" s="20"/>
-      <c r="G18" s="20"/>
-      <c r="H18" s="20"/>
+    </row>
+    <row r="18" spans="1:9">
+      <c r="A18" s="21"/>
+      <c r="B18" s="21"/>
+      <c r="C18" s="21"/>
+      <c r="D18" s="21"/>
+      <c r="E18" s="23"/>
+      <c r="F18" s="21"/>
+      <c r="G18" s="21"/>
+      <c r="H18" s="7"/>
       <c r="I18" s="7"/>
-      <c r="J18" s="7"/>
-    </row>
-    <row r="19" spans="1:10">
-      <c r="A19" s="20"/>
-      <c r="B19" s="20"/>
-      <c r="C19" s="20"/>
-      <c r="D19" s="20"/>
-      <c r="E19" s="23"/>
-      <c r="F19" s="20"/>
-      <c r="G19" s="20"/>
-      <c r="H19" s="20"/>
+    </row>
+    <row r="19" spans="1:9">
+      <c r="A19" s="21"/>
+      <c r="B19" s="21"/>
+      <c r="C19" s="21"/>
+      <c r="D19" s="21"/>
+      <c r="E19" s="24"/>
+      <c r="F19" s="21"/>
+      <c r="G19" s="21"/>
+      <c r="H19" s="7"/>
       <c r="I19" s="7"/>
-      <c r="J19" s="7"/>
-    </row>
-    <row r="20" spans="1:10">
-      <c r="A20" s="20"/>
-      <c r="B20" s="20"/>
-      <c r="C20" s="20"/>
-      <c r="D20" s="20"/>
-      <c r="E20" s="23"/>
-      <c r="F20" s="20"/>
-      <c r="G20" s="20"/>
-      <c r="H20" s="20"/>
+    </row>
+    <row r="20" spans="1:9">
+      <c r="A20" s="21"/>
+      <c r="B20" s="21"/>
+      <c r="C20" s="21"/>
+      <c r="D20" s="21"/>
+      <c r="E20" s="24"/>
+      <c r="F20" s="21"/>
+      <c r="G20" s="21"/>
+      <c r="H20" s="7"/>
       <c r="I20" s="7"/>
-      <c r="J20" s="7"/>
-    </row>
-    <row r="21" spans="1:10">
-      <c r="A21" s="20"/>
-      <c r="B21" s="20"/>
-      <c r="C21" s="20"/>
-      <c r="D21" s="20"/>
-      <c r="E21" s="23"/>
-      <c r="F21" s="20"/>
-      <c r="G21" s="20"/>
-      <c r="H21" s="20"/>
+    </row>
+    <row r="21" spans="1:9">
+      <c r="A21" s="21"/>
+      <c r="B21" s="21"/>
+      <c r="C21" s="21"/>
+      <c r="D21" s="21"/>
+      <c r="E21" s="24"/>
+      <c r="F21" s="21"/>
+      <c r="G21" s="21"/>
+      <c r="H21" s="7"/>
       <c r="I21" s="7"/>
-      <c r="J21" s="7"/>
-    </row>
-    <row r="22" spans="1:10">
-      <c r="A22" s="20"/>
-      <c r="B22" s="20"/>
-      <c r="C22" s="20"/>
-      <c r="D22" s="20"/>
-      <c r="E22" s="24"/>
-      <c r="F22" s="20"/>
-      <c r="G22" s="20"/>
-      <c r="H22" s="20"/>
+    </row>
+    <row r="22" spans="1:9">
+      <c r="A22" s="21"/>
+      <c r="B22" s="21"/>
+      <c r="C22" s="21"/>
+      <c r="D22" s="21"/>
+      <c r="E22" s="25"/>
+      <c r="F22" s="21"/>
+      <c r="G22" s="21"/>
+      <c r="H22" s="7"/>
       <c r="I22" s="7"/>
-      <c r="J22" s="7"/>
     </row>
   </sheetData>
-  <mergeCells count="33">
-    <mergeCell ref="A1:H1"/>
+  <mergeCells count="29">
+    <mergeCell ref="A1:G1"/>
     <mergeCell ref="A3:A7"/>
     <mergeCell ref="A8:A12"/>
     <mergeCell ref="A13:A17"/>
@@ -2114,10 +2080,6 @@
     <mergeCell ref="G8:G12"/>
     <mergeCell ref="G13:G17"/>
     <mergeCell ref="G18:G22"/>
-    <mergeCell ref="H3:H7"/>
-    <mergeCell ref="H8:H12"/>
-    <mergeCell ref="H13:H17"/>
-    <mergeCell ref="H18:H22"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E3:E22">
@@ -2132,86 +2094,75 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:F30"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4" outlineLevelCol="5"/>
+  <dimension ref="A1:E30"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4" outlineLevelCol="4"/>
   <cols>
     <col min="1" max="1" width="21.6666666666667" style="14" customWidth="1"/>
     <col min="2" max="2" width="22.1111111111111" style="14" customWidth="1"/>
     <col min="3" max="3" width="45.8888888888889" style="14" customWidth="1"/>
     <col min="4" max="4" width="22.1111111111111" style="14" customWidth="1"/>
     <col min="5" max="5" width="23.1111111111111" style="14" customWidth="1"/>
-    <col min="6" max="6" width="15" style="14" customWidth="1"/>
-    <col min="7" max="16384" width="9" style="14"/>
+    <col min="6" max="16384" width="9" style="14"/>
   </cols>
   <sheetData>
-    <row r="1" ht="20" customHeight="1" spans="1:6">
+    <row r="1" ht="20" customHeight="1" spans="1:5">
       <c r="A1" s="15" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="B1" s="15"/>
       <c r="C1" s="15"/>
       <c r="D1" s="15"/>
       <c r="E1" s="15"/>
-      <c r="F1" s="15"/>
-    </row>
-    <row r="2" s="13" customFormat="1" ht="30" customHeight="1" spans="1:6">
+    </row>
+    <row r="2" s="13" customFormat="1" ht="30" customHeight="1" spans="1:5">
       <c r="A2" s="16" t="s">
         <v>20</v>
       </c>
       <c r="B2" s="16" t="s">
+        <v>37</v>
+      </c>
+      <c r="C2" s="16" t="s">
+        <v>38</v>
+      </c>
+      <c r="D2" s="16" t="s">
         <v>39</v>
       </c>
-      <c r="C2" s="16" t="s">
+      <c r="E2" s="16" t="s">
         <v>40</v>
       </c>
-      <c r="D2" s="16" t="s">
+    </row>
+    <row r="3" ht="20" customHeight="1" spans="1:5">
+      <c r="A3" s="9" t="s">
+        <v>27</v>
+      </c>
+      <c r="B3" s="9" t="s">
         <v>41</v>
       </c>
-      <c r="E2" s="16" t="s">
+      <c r="C3" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="F2" s="16" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="3" ht="20" customHeight="1" spans="1:6">
-      <c r="A3" s="9" t="s">
-        <v>28</v>
-      </c>
-      <c r="B3" s="9" t="s">
+      <c r="D3" s="17" t="s">
         <v>43</v>
-      </c>
-      <c r="C3" s="9" t="s">
-        <v>44</v>
-      </c>
-      <c r="D3" s="17" t="s">
-        <v>45</v>
       </c>
       <c r="E3" s="9">
         <v>1</v>
       </c>
-      <c r="F3" s="9" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="4" ht="20" customHeight="1" spans="1:6">
+    </row>
+    <row r="4" ht="20" customHeight="1" spans="1:5">
       <c r="A4" s="9" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="D4" s="17" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="E4" s="9">
         <v>2</v>
-      </c>
-      <c r="F4" s="9" t="s">
-        <v>34</v>
       </c>
     </row>
     <row r="5" ht="20" customHeight="1"/>
@@ -2242,7 +2193,7 @@
     <row r="30" ht="20" customHeight="1"/>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A1:E1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>
@@ -2252,7 +2203,7 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:O16"/>
+  <dimension ref="A1:N16"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.8"/>
   <cols>
     <col min="1" max="1" width="15.2222222222222" style="9" customWidth="1"/>
@@ -2269,13 +2220,12 @@
     <col min="12" max="12" width="19.7777777777778" style="9" customWidth="1"/>
     <col min="13" max="13" width="25.2222222222222" style="9" customWidth="1"/>
     <col min="14" max="14" width="27.4444444444444" style="9" customWidth="1"/>
-    <col min="15" max="15" width="13" style="9" customWidth="1"/>
-    <col min="16" max="16384" width="9" style="9"/>
+    <col min="15" max="16384" width="9" style="9"/>
   </cols>
   <sheetData>
-    <row r="1" ht="22.8" spans="1:15">
+    <row r="1" ht="22.8" spans="1:14">
       <c r="A1" s="10" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="B1" s="11"/>
       <c r="C1" s="11"/>
@@ -2290,132 +2240,125 @@
       <c r="L1" s="11"/>
       <c r="M1" s="11"/>
       <c r="N1" s="11"/>
-      <c r="O1" s="11"/>
-    </row>
-    <row r="2" s="8" customFormat="1" ht="30" customHeight="1" spans="1:15">
+    </row>
+    <row r="2" s="8" customFormat="1" ht="30" customHeight="1" spans="1:14">
       <c r="A2" s="5" t="s">
         <v>20</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C2" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="D2" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="E2" s="5" t="s">
         <v>49</v>
       </c>
-      <c r="D2" s="5" t="s">
+      <c r="F2" s="5" t="s">
         <v>50</v>
       </c>
-      <c r="E2" s="5" t="s">
+      <c r="G2" s="5" t="s">
         <v>51</v>
       </c>
-      <c r="F2" s="5" t="s">
+      <c r="H2" s="5" t="s">
         <v>52</v>
       </c>
-      <c r="G2" s="5" t="s">
+      <c r="I2" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="H2" s="5" t="s">
+      <c r="J2" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="I2" s="5" t="s">
+      <c r="K2" s="5" t="s">
         <v>55</v>
       </c>
-      <c r="J2" s="5" t="s">
+      <c r="L2" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="K2" s="5" t="s">
+      <c r="M2" s="5" t="s">
         <v>57</v>
       </c>
-      <c r="L2" s="5" t="s">
+      <c r="N2" s="5" t="s">
         <v>58</v>
       </c>
-      <c r="M2" s="5" t="s">
+    </row>
+    <row r="3" ht="20" customHeight="1" spans="1:14">
+      <c r="A3" s="12" t="s">
+        <v>27</v>
+      </c>
+      <c r="B3" s="12" t="s">
+        <v>41</v>
+      </c>
+      <c r="C3" s="12" t="s">
         <v>59</v>
       </c>
-      <c r="N2" s="5" t="s">
+      <c r="D3" s="12" t="s">
         <v>60</v>
-      </c>
-      <c r="O2" s="5" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="3" ht="20" customHeight="1" spans="1:15">
-      <c r="A3" s="12" t="s">
-        <v>28</v>
-      </c>
-      <c r="B3" s="12" t="s">
-        <v>43</v>
-      </c>
-      <c r="C3" s="12" t="s">
-        <v>61</v>
-      </c>
-      <c r="D3" s="12" t="s">
-        <v>62</v>
       </c>
       <c r="E3" s="12">
         <v>1</v>
       </c>
       <c r="F3" s="12" t="s">
+        <v>61</v>
+      </c>
+      <c r="G3" s="12" t="s">
+        <v>62</v>
+      </c>
+      <c r="H3" s="12" t="s">
         <v>63</v>
       </c>
-      <c r="G3" s="12" t="s">
+      <c r="I3" s="12" t="s">
+        <v>63</v>
+      </c>
+      <c r="J3" s="12" t="s">
+        <v>63</v>
+      </c>
+      <c r="K3" s="12" t="s">
+        <v>63</v>
+      </c>
+      <c r="L3" s="12" t="s">
+        <v>63</v>
+      </c>
+      <c r="M3" s="12" t="s">
         <v>64</v>
-      </c>
-      <c r="H3" s="12" t="s">
-        <v>65</v>
-      </c>
-      <c r="I3" s="12" t="s">
-        <v>65</v>
-      </c>
-      <c r="J3" s="12" t="s">
-        <v>65</v>
-      </c>
-      <c r="K3" s="12" t="s">
-        <v>65</v>
-      </c>
-      <c r="L3" s="12" t="s">
-        <v>65</v>
-      </c>
-      <c r="M3" s="12" t="s">
-        <v>66</v>
       </c>
       <c r="N3" s="12">
         <v>10</v>
       </c>
-      <c r="O3" s="12" t="s">
+    </row>
+    <row r="4" ht="20" customHeight="1" spans="1:14">
+      <c r="A4" s="12" t="s">
+        <v>27</v>
+      </c>
+      <c r="B4" s="12" t="s">
+        <v>41</v>
+      </c>
+      <c r="C4" s="12" t="s">
         <v>65</v>
       </c>
-    </row>
-    <row r="4" ht="20" customHeight="1" spans="1:15">
-      <c r="A4" s="12" t="s">
-        <v>28</v>
-      </c>
-      <c r="B4" s="12" t="s">
-        <v>43</v>
-      </c>
-      <c r="C4" s="12" t="s">
-        <v>67</v>
-      </c>
       <c r="D4" s="12" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="E4" s="12">
         <v>2</v>
       </c>
       <c r="F4" s="12" t="s">
+        <v>67</v>
+      </c>
+      <c r="G4" s="12" t="s">
+        <v>63</v>
+      </c>
+      <c r="H4" s="12" t="s">
+        <v>63</v>
+      </c>
+      <c r="I4" s="12" t="s">
+        <v>68</v>
+      </c>
+      <c r="J4" s="12" t="s">
         <v>69</v>
-      </c>
-      <c r="G4" s="12" t="s">
-        <v>65</v>
-      </c>
-      <c r="H4" s="12" t="s">
-        <v>65</v>
-      </c>
-      <c r="I4" s="12" t="s">
-        <v>70</v>
-      </c>
-      <c r="J4" s="12" t="s">
-        <v>71</v>
       </c>
       <c r="K4" s="12">
         <v>360</v>
@@ -2424,63 +2367,57 @@
         <v>104857600</v>
       </c>
       <c r="M4" s="12" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="N4" s="12">
         <v>15</v>
       </c>
-      <c r="O4" s="12" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="5" ht="20" customHeight="1" spans="1:15">
+    </row>
+    <row r="5" ht="20" customHeight="1" spans="1:14">
       <c r="A5" s="12" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B5" s="12" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="C5" s="12" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="D5" s="12" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="E5" s="12">
         <v>1</v>
       </c>
       <c r="F5" s="12" t="s">
+        <v>61</v>
+      </c>
+      <c r="G5" s="12" t="s">
+        <v>73</v>
+      </c>
+      <c r="H5" s="12" t="s">
         <v>63</v>
       </c>
-      <c r="G5" s="12" t="s">
-        <v>75</v>
-      </c>
-      <c r="H5" s="12" t="s">
-        <v>65</v>
-      </c>
       <c r="I5" s="12" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="J5" s="12" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="K5" s="12" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="L5" s="12" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="M5" s="12" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="N5" s="12">
         <v>20</v>
       </c>
-      <c r="O5" s="12" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="6" ht="20" customHeight="1" spans="1:15">
+    </row>
+    <row r="6" ht="20" customHeight="1" spans="1:14">
       <c r="A6" s="12"/>
       <c r="B6" s="12"/>
       <c r="C6" s="12"/>
@@ -2495,9 +2432,8 @@
       <c r="L6" s="12"/>
       <c r="M6" s="12"/>
       <c r="N6" s="12"/>
-      <c r="O6" s="12"/>
-    </row>
-    <row r="7" ht="20" customHeight="1" spans="1:15">
+    </row>
+    <row r="7" ht="20" customHeight="1" spans="1:14">
       <c r="A7" s="12"/>
       <c r="B7" s="12"/>
       <c r="C7" s="12"/>
@@ -2512,9 +2448,8 @@
       <c r="L7" s="12"/>
       <c r="M7" s="12"/>
       <c r="N7" s="12"/>
-      <c r="O7" s="12"/>
-    </row>
-    <row r="8" ht="20" customHeight="1" spans="1:15">
+    </row>
+    <row r="8" ht="20" customHeight="1" spans="1:14">
       <c r="A8" s="12"/>
       <c r="B8" s="12"/>
       <c r="C8" s="12"/>
@@ -2529,9 +2464,8 @@
       <c r="L8" s="12"/>
       <c r="M8" s="12"/>
       <c r="N8" s="12"/>
-      <c r="O8" s="12"/>
-    </row>
-    <row r="9" ht="20" customHeight="1" spans="1:15">
+    </row>
+    <row r="9" ht="20" customHeight="1" spans="1:14">
       <c r="A9" s="12"/>
       <c r="B9" s="12"/>
       <c r="C9" s="12"/>
@@ -2546,9 +2480,8 @@
       <c r="L9" s="12"/>
       <c r="M9" s="12"/>
       <c r="N9" s="12"/>
-      <c r="O9" s="12"/>
-    </row>
-    <row r="10" ht="20" customHeight="1" spans="1:15">
+    </row>
+    <row r="10" ht="20" customHeight="1" spans="1:14">
       <c r="A10" s="12"/>
       <c r="B10" s="12"/>
       <c r="C10" s="12"/>
@@ -2563,9 +2496,8 @@
       <c r="L10" s="12"/>
       <c r="M10" s="12"/>
       <c r="N10" s="12"/>
-      <c r="O10" s="12"/>
-    </row>
-    <row r="11" ht="20" customHeight="1" spans="1:15">
+    </row>
+    <row r="11" ht="20" customHeight="1" spans="1:14">
       <c r="A11" s="12"/>
       <c r="B11" s="12"/>
       <c r="C11" s="12"/>
@@ -2580,9 +2512,8 @@
       <c r="L11" s="12"/>
       <c r="M11" s="12"/>
       <c r="N11" s="12"/>
-      <c r="O11" s="12"/>
-    </row>
-    <row r="12" ht="20" customHeight="1" spans="1:15">
+    </row>
+    <row r="12" ht="20" customHeight="1" spans="1:14">
       <c r="A12" s="12"/>
       <c r="B12" s="12"/>
       <c r="C12" s="12"/>
@@ -2597,9 +2528,8 @@
       <c r="L12" s="12"/>
       <c r="M12" s="12"/>
       <c r="N12" s="12"/>
-      <c r="O12" s="12"/>
-    </row>
-    <row r="13" ht="20" customHeight="1" spans="1:15">
+    </row>
+    <row r="13" ht="20" customHeight="1" spans="1:14">
       <c r="A13" s="12"/>
       <c r="B13" s="12"/>
       <c r="C13" s="12"/>
@@ -2614,9 +2544,8 @@
       <c r="L13" s="12"/>
       <c r="M13" s="12"/>
       <c r="N13" s="12"/>
-      <c r="O13" s="12"/>
-    </row>
-    <row r="14" ht="20" customHeight="1" spans="1:15">
+    </row>
+    <row r="14" ht="20" customHeight="1" spans="1:14">
       <c r="A14" s="12"/>
       <c r="B14" s="12"/>
       <c r="C14" s="12"/>
@@ -2631,9 +2560,8 @@
       <c r="L14" s="12"/>
       <c r="M14" s="12"/>
       <c r="N14" s="12"/>
-      <c r="O14" s="12"/>
-    </row>
-    <row r="15" ht="20" customHeight="1" spans="1:15">
+    </row>
+    <row r="15" ht="20" customHeight="1" spans="1:14">
       <c r="A15" s="12"/>
       <c r="B15" s="12"/>
       <c r="C15" s="12"/>
@@ -2648,9 +2576,8 @@
       <c r="L15" s="12"/>
       <c r="M15" s="12"/>
       <c r="N15" s="12"/>
-      <c r="O15" s="12"/>
-    </row>
-    <row r="16" ht="20" customHeight="1" spans="1:15">
+    </row>
+    <row r="16" ht="20" customHeight="1" spans="1:14">
       <c r="A16" s="12"/>
       <c r="B16" s="12"/>
       <c r="C16" s="12"/>
@@ -2665,11 +2592,10 @@
       <c r="L16" s="12"/>
       <c r="M16" s="12"/>
       <c r="N16" s="12"/>
-      <c r="O16" s="12"/>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:O1"/>
+    <mergeCell ref="A1:N1"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="F3:F5">
@@ -2701,7 +2627,7 @@
     <row r="1" ht="23.4" spans="4:16">
       <c r="D1" s="4"/>
       <c r="E1" s="4" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="F1" s="4"/>
       <c r="G1" s="4"/>
@@ -2720,43 +2646,43 @@
         <v>20</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C2" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="D2" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="E2" s="6" t="s">
+        <v>77</v>
+      </c>
+      <c r="F2" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="G2" s="6" t="s">
+        <v>79</v>
+      </c>
+      <c r="H2" s="6" t="s">
+        <v>80</v>
+      </c>
+      <c r="I2" s="6" t="s">
+        <v>81</v>
+      </c>
+      <c r="J2" s="6" t="s">
+        <v>82</v>
+      </c>
+      <c r="K2" s="6" t="s">
+        <v>83</v>
+      </c>
+      <c r="L2" s="6" t="s">
+        <v>84</v>
+      </c>
+      <c r="M2" s="6" t="s">
         <v>49</v>
       </c>
-      <c r="D2" s="6" t="s">
-        <v>78</v>
-      </c>
-      <c r="E2" s="6" t="s">
-        <v>79</v>
-      </c>
-      <c r="F2" s="6" t="s">
-        <v>80</v>
-      </c>
-      <c r="G2" s="6" t="s">
-        <v>81</v>
-      </c>
-      <c r="H2" s="6" t="s">
-        <v>82</v>
-      </c>
-      <c r="I2" s="6" t="s">
-        <v>83</v>
-      </c>
-      <c r="J2" s="6" t="s">
-        <v>84</v>
-      </c>
-      <c r="K2" s="6" t="s">
+      <c r="N2" s="6" t="s">
         <v>85</v>
-      </c>
-      <c r="L2" s="6" t="s">
-        <v>86</v>
-      </c>
-      <c r="M2" s="6" t="s">
-        <v>51</v>
-      </c>
-      <c r="N2" s="6" t="s">
-        <v>87</v>
       </c>
       <c r="O2" s="6" t="s">
         <v>24</v>
@@ -2812,7 +2738,7 @@
   <sheetData>
     <row r="1" s="1" customFormat="1" ht="30" customHeight="1" spans="1:2">
       <c r="A1" s="2" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>22</v>
@@ -2823,47 +2749,47 @@
         <v>20</v>
       </c>
       <c r="B2" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
     </row>
     <row r="3" ht="20" customHeight="1" spans="1:2">
       <c r="A3" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="B3" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
     </row>
     <row r="4" ht="20" customHeight="1" spans="1:2">
       <c r="A4" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="B4" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
     </row>
     <row r="5" ht="20" customHeight="1" spans="1:2">
       <c r="A5" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="B5" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1" spans="1:2">
       <c r="A6" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="B6" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
     </row>
     <row r="7" ht="20" customHeight="1" spans="1:2">
       <c r="A7" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="B7" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: implement course bulk import service, add frontend integration, and include Excel template
</commit_message>
<xml_diff>
--- a/doc/templates/Hango_Course_Import_Template.xlsx
+++ b/doc/templates/Hango_Course_Import_Template.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="23040" windowHeight="8987" activeTab="1"/>
+    <workbookView windowWidth="23028" windowHeight="9720" activeTab="3"/>
   </bookViews>
   <sheets>
     <sheet name="README_AND_RULES" sheetId="1" r:id="rId1"/>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="133" uniqueCount="95">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="132" uniqueCount="94">
   <si>
     <t>Hango Course Import Template - Rules</t>
   </si>
@@ -107,9 +107,6 @@
   </si>
   <si>
     <t>Difficulty</t>
-  </si>
-  <si>
-    <t>Price</t>
   </si>
   <si>
     <t>Thumbnail URL</t>
@@ -1160,6 +1157,9 @@
     <xf numFmtId="0" fontId="9" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
@@ -1174,9 +1174,6 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="10" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
@@ -1751,19 +1748,18 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:I22"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4"/>
+  <dimension ref="A1:H22"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4" outlineLevelCol="7"/>
   <cols>
     <col min="1" max="1" width="21.6666666666667" customWidth="1"/>
     <col min="2" max="2" width="30.6666666666667" customWidth="1"/>
     <col min="3" max="3" width="64.4444444444444" customWidth="1"/>
     <col min="4" max="4" width="13.8888888888889" customWidth="1"/>
     <col min="5" max="5" width="10.7777777777778" customWidth="1"/>
-    <col min="6" max="6" width="8.33333333333333" customWidth="1"/>
-    <col min="7" max="7" width="31.5555555555556" customWidth="1"/>
+    <col min="6" max="6" width="31.5555555555556" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="22.8" spans="1:9">
+    <row r="1" ht="22.8" spans="1:8">
       <c r="A1" s="18" t="s">
         <v>19</v>
       </c>
@@ -1772,11 +1768,10 @@
       <c r="D1" s="19"/>
       <c r="E1" s="19"/>
       <c r="F1" s="19"/>
-      <c r="G1" s="19"/>
+      <c r="G1" s="7"/>
       <c r="H1" s="7"/>
-      <c r="I1" s="7"/>
-    </row>
-    <row r="2" s="13" customFormat="1" ht="30" customHeight="1" spans="1:9">
+    </row>
+    <row r="2" s="13" customFormat="1" ht="30" customHeight="1" spans="1:8">
       <c r="A2" s="5" t="s">
         <v>20</v>
       </c>
@@ -1795,263 +1790,236 @@
       <c r="F2" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="G2" s="5" t="s">
+      <c r="G2" s="20"/>
+      <c r="H2" s="21"/>
+    </row>
+    <row r="3" spans="1:8">
+      <c r="A3" s="22" t="s">
         <v>26</v>
       </c>
-      <c r="H2" s="20"/>
-      <c r="I2" s="26"/>
-    </row>
-    <row r="3" spans="1:9">
-      <c r="A3" s="21" t="s">
+      <c r="B3" s="22" t="s">
         <v>27</v>
       </c>
-      <c r="B3" s="21" t="s">
+      <c r="C3" s="22" t="s">
         <v>28</v>
       </c>
-      <c r="C3" s="21" t="s">
+      <c r="D3" s="22" t="s">
         <v>29</v>
       </c>
-      <c r="D3" s="21" t="s">
+      <c r="E3" s="23" t="s">
         <v>30</v>
       </c>
-      <c r="E3" s="22" t="s">
+      <c r="F3" s="22" t="s">
         <v>31</v>
       </c>
-      <c r="F3" s="21">
-        <v>0</v>
-      </c>
-      <c r="G3" s="21" t="s">
+      <c r="G3" s="7"/>
+      <c r="H3" s="7"/>
+    </row>
+    <row r="4" spans="1:8">
+      <c r="A4" s="22"/>
+      <c r="B4" s="22"/>
+      <c r="C4" s="22"/>
+      <c r="D4" s="22"/>
+      <c r="E4" s="23"/>
+      <c r="F4" s="22"/>
+      <c r="G4" s="7"/>
+      <c r="H4" s="7"/>
+    </row>
+    <row r="5" spans="1:8">
+      <c r="A5" s="22"/>
+      <c r="B5" s="22"/>
+      <c r="C5" s="22"/>
+      <c r="D5" s="22"/>
+      <c r="E5" s="23"/>
+      <c r="F5" s="22"/>
+      <c r="G5" s="7"/>
+      <c r="H5" s="7"/>
+    </row>
+    <row r="6" spans="1:8">
+      <c r="A6" s="22"/>
+      <c r="B6" s="22"/>
+      <c r="C6" s="22"/>
+      <c r="D6" s="22"/>
+      <c r="E6" s="23"/>
+      <c r="F6" s="22"/>
+      <c r="G6" s="7"/>
+      <c r="H6" s="7"/>
+    </row>
+    <row r="7" spans="1:8">
+      <c r="A7" s="22"/>
+      <c r="B7" s="22"/>
+      <c r="C7" s="22"/>
+      <c r="D7" s="22"/>
+      <c r="E7" s="23"/>
+      <c r="F7" s="22"/>
+      <c r="G7" s="7"/>
+      <c r="H7" s="7"/>
+    </row>
+    <row r="8" spans="1:8">
+      <c r="A8" s="22" t="s">
         <v>32</v>
       </c>
-      <c r="H3" s="7"/>
-      <c r="I3" s="7"/>
-    </row>
-    <row r="4" spans="1:9">
-      <c r="A4" s="21"/>
-      <c r="B4" s="21"/>
-      <c r="C4" s="21"/>
-      <c r="D4" s="21"/>
-      <c r="E4" s="22"/>
-      <c r="F4" s="21"/>
-      <c r="G4" s="21"/>
-      <c r="H4" s="7"/>
-      <c r="I4" s="7"/>
-    </row>
-    <row r="5" spans="1:9">
-      <c r="A5" s="21"/>
-      <c r="B5" s="21"/>
-      <c r="C5" s="21"/>
-      <c r="D5" s="21"/>
-      <c r="E5" s="22"/>
-      <c r="F5" s="21"/>
-      <c r="G5" s="21"/>
-      <c r="H5" s="7"/>
-      <c r="I5" s="7"/>
-    </row>
-    <row r="6" spans="1:9">
-      <c r="A6" s="21"/>
-      <c r="B6" s="21"/>
-      <c r="C6" s="21"/>
-      <c r="D6" s="21"/>
-      <c r="E6" s="22"/>
-      <c r="F6" s="21"/>
-      <c r="G6" s="21"/>
-      <c r="H6" s="7"/>
-      <c r="I6" s="7"/>
-    </row>
-    <row r="7" spans="1:9">
-      <c r="A7" s="21"/>
-      <c r="B7" s="21"/>
-      <c r="C7" s="21"/>
-      <c r="D7" s="21"/>
-      <c r="E7" s="22"/>
-      <c r="F7" s="21"/>
-      <c r="G7" s="21"/>
-      <c r="H7" s="7"/>
-      <c r="I7" s="7"/>
-    </row>
-    <row r="8" spans="1:9">
-      <c r="A8" s="21" t="s">
+      <c r="B8" s="22" t="s">
         <v>33</v>
       </c>
-      <c r="B8" s="21" t="s">
+      <c r="C8" s="22" t="s">
         <v>34</v>
       </c>
-      <c r="C8" s="21" t="s">
-        <v>35</v>
-      </c>
-      <c r="D8" s="21" t="s">
+      <c r="D8" s="22" t="s">
+        <v>29</v>
+      </c>
+      <c r="E8" s="23" t="s">
         <v>30</v>
       </c>
-      <c r="E8" s="22" t="s">
+      <c r="F8" s="22" t="s">
         <v>31</v>
       </c>
-      <c r="F8" s="21">
-        <v>0</v>
-      </c>
-      <c r="G8" s="21" t="s">
-        <v>32</v>
-      </c>
+      <c r="G8" s="7"/>
       <c r="H8" s="7"/>
-      <c r="I8" s="7"/>
-    </row>
-    <row r="9" spans="1:9">
-      <c r="A9" s="21"/>
-      <c r="B9" s="21"/>
-      <c r="C9" s="21"/>
-      <c r="D9" s="21"/>
-      <c r="E9" s="22"/>
-      <c r="F9" s="21"/>
-      <c r="G9" s="21"/>
+    </row>
+    <row r="9" spans="1:8">
+      <c r="A9" s="22"/>
+      <c r="B9" s="22"/>
+      <c r="C9" s="22"/>
+      <c r="D9" s="22"/>
+      <c r="E9" s="23"/>
+      <c r="F9" s="22"/>
+      <c r="G9" s="7"/>
       <c r="H9" s="7"/>
-      <c r="I9" s="7"/>
-    </row>
-    <row r="10" spans="1:9">
-      <c r="A10" s="21"/>
-      <c r="B10" s="21"/>
-      <c r="C10" s="21"/>
-      <c r="D10" s="21"/>
-      <c r="E10" s="22"/>
-      <c r="F10" s="21"/>
-      <c r="G10" s="21"/>
+    </row>
+    <row r="10" spans="1:8">
+      <c r="A10" s="22"/>
+      <c r="B10" s="22"/>
+      <c r="C10" s="22"/>
+      <c r="D10" s="22"/>
+      <c r="E10" s="23"/>
+      <c r="F10" s="22"/>
+      <c r="G10" s="7"/>
       <c r="H10" s="7"/>
-      <c r="I10" s="7"/>
-    </row>
-    <row r="11" spans="1:9">
-      <c r="A11" s="21"/>
-      <c r="B11" s="21"/>
-      <c r="C11" s="21"/>
-      <c r="D11" s="21"/>
-      <c r="E11" s="22"/>
-      <c r="F11" s="21"/>
-      <c r="G11" s="21"/>
+    </row>
+    <row r="11" spans="1:8">
+      <c r="A11" s="22"/>
+      <c r="B11" s="22"/>
+      <c r="C11" s="22"/>
+      <c r="D11" s="22"/>
+      <c r="E11" s="23"/>
+      <c r="F11" s="22"/>
+      <c r="G11" s="7"/>
       <c r="H11" s="7"/>
-      <c r="I11" s="7"/>
-    </row>
-    <row r="12" spans="1:9">
-      <c r="A12" s="21"/>
-      <c r="B12" s="21"/>
-      <c r="C12" s="21"/>
-      <c r="D12" s="21"/>
-      <c r="E12" s="22"/>
-      <c r="F12" s="21"/>
-      <c r="G12" s="21"/>
+    </row>
+    <row r="12" spans="1:8">
+      <c r="A12" s="22"/>
+      <c r="B12" s="22"/>
+      <c r="C12" s="22"/>
+      <c r="D12" s="22"/>
+      <c r="E12" s="23"/>
+      <c r="F12" s="22"/>
+      <c r="G12" s="7"/>
       <c r="H12" s="7"/>
-      <c r="I12" s="7"/>
-    </row>
-    <row r="13" spans="1:9">
-      <c r="A13" s="21"/>
-      <c r="B13" s="21"/>
-      <c r="C13" s="21"/>
-      <c r="D13" s="21"/>
-      <c r="E13" s="23"/>
-      <c r="F13" s="21"/>
-      <c r="G13" s="21"/>
+    </row>
+    <row r="13" spans="1:8">
+      <c r="A13" s="22"/>
+      <c r="B13" s="22"/>
+      <c r="C13" s="22"/>
+      <c r="D13" s="22"/>
+      <c r="E13" s="24"/>
+      <c r="F13" s="22"/>
+      <c r="G13" s="7"/>
       <c r="H13" s="7"/>
-      <c r="I13" s="7"/>
-    </row>
-    <row r="14" spans="1:9">
-      <c r="A14" s="21"/>
-      <c r="B14" s="21"/>
-      <c r="C14" s="21"/>
-      <c r="D14" s="21"/>
-      <c r="E14" s="24"/>
-      <c r="F14" s="21"/>
-      <c r="G14" s="21"/>
+    </row>
+    <row r="14" spans="1:8">
+      <c r="A14" s="22"/>
+      <c r="B14" s="22"/>
+      <c r="C14" s="22"/>
+      <c r="D14" s="22"/>
+      <c r="E14" s="25"/>
+      <c r="F14" s="22"/>
+      <c r="G14" s="7"/>
       <c r="H14" s="7"/>
-      <c r="I14" s="7"/>
-    </row>
-    <row r="15" spans="1:9">
-      <c r="A15" s="21"/>
-      <c r="B15" s="21"/>
-      <c r="C15" s="21"/>
-      <c r="D15" s="21"/>
-      <c r="E15" s="24"/>
-      <c r="F15" s="21"/>
-      <c r="G15" s="21"/>
+    </row>
+    <row r="15" spans="1:8">
+      <c r="A15" s="22"/>
+      <c r="B15" s="22"/>
+      <c r="C15" s="22"/>
+      <c r="D15" s="22"/>
+      <c r="E15" s="25"/>
+      <c r="F15" s="22"/>
+      <c r="G15" s="7"/>
       <c r="H15" s="7"/>
-      <c r="I15" s="7"/>
-    </row>
-    <row r="16" ht="12" customHeight="1" spans="1:9">
-      <c r="A16" s="21"/>
-      <c r="B16" s="21"/>
-      <c r="C16" s="21"/>
-      <c r="D16" s="21"/>
-      <c r="E16" s="24"/>
-      <c r="F16" s="21"/>
-      <c r="G16" s="21"/>
+    </row>
+    <row r="16" ht="12" customHeight="1" spans="1:8">
+      <c r="A16" s="22"/>
+      <c r="B16" s="22"/>
+      <c r="C16" s="22"/>
+      <c r="D16" s="22"/>
+      <c r="E16" s="25"/>
+      <c r="F16" s="22"/>
+      <c r="G16" s="7"/>
       <c r="H16" s="7"/>
-      <c r="I16" s="7"/>
-    </row>
-    <row r="17" spans="1:9">
-      <c r="A17" s="21"/>
-      <c r="B17" s="21"/>
-      <c r="C17" s="21"/>
-      <c r="D17" s="21"/>
-      <c r="E17" s="25"/>
-      <c r="F17" s="21"/>
-      <c r="G17" s="21"/>
+    </row>
+    <row r="17" spans="1:8">
+      <c r="A17" s="22"/>
+      <c r="B17" s="22"/>
+      <c r="C17" s="22"/>
+      <c r="D17" s="22"/>
+      <c r="E17" s="26"/>
+      <c r="F17" s="22"/>
+      <c r="G17" s="7"/>
       <c r="H17" s="7"/>
-      <c r="I17" s="7"/>
-    </row>
-    <row r="18" spans="1:9">
-      <c r="A18" s="21"/>
-      <c r="B18" s="21"/>
-      <c r="C18" s="21"/>
-      <c r="D18" s="21"/>
-      <c r="E18" s="23"/>
-      <c r="F18" s="21"/>
-      <c r="G18" s="21"/>
+    </row>
+    <row r="18" spans="1:8">
+      <c r="A18" s="22"/>
+      <c r="B18" s="22"/>
+      <c r="C18" s="22"/>
+      <c r="D18" s="22"/>
+      <c r="E18" s="24"/>
+      <c r="F18" s="22"/>
+      <c r="G18" s="7"/>
       <c r="H18" s="7"/>
-      <c r="I18" s="7"/>
-    </row>
-    <row r="19" spans="1:9">
-      <c r="A19" s="21"/>
-      <c r="B19" s="21"/>
-      <c r="C19" s="21"/>
-      <c r="D19" s="21"/>
-      <c r="E19" s="24"/>
-      <c r="F19" s="21"/>
-      <c r="G19" s="21"/>
+    </row>
+    <row r="19" spans="1:8">
+      <c r="A19" s="22"/>
+      <c r="B19" s="22"/>
+      <c r="C19" s="22"/>
+      <c r="D19" s="22"/>
+      <c r="E19" s="25"/>
+      <c r="F19" s="22"/>
+      <c r="G19" s="7"/>
       <c r="H19" s="7"/>
-      <c r="I19" s="7"/>
-    </row>
-    <row r="20" spans="1:9">
-      <c r="A20" s="21"/>
-      <c r="B20" s="21"/>
-      <c r="C20" s="21"/>
-      <c r="D20" s="21"/>
-      <c r="E20" s="24"/>
-      <c r="F20" s="21"/>
-      <c r="G20" s="21"/>
+    </row>
+    <row r="20" spans="1:8">
+      <c r="A20" s="22"/>
+      <c r="B20" s="22"/>
+      <c r="C20" s="22"/>
+      <c r="D20" s="22"/>
+      <c r="E20" s="25"/>
+      <c r="F20" s="22"/>
+      <c r="G20" s="7"/>
       <c r="H20" s="7"/>
-      <c r="I20" s="7"/>
-    </row>
-    <row r="21" spans="1:9">
-      <c r="A21" s="21"/>
-      <c r="B21" s="21"/>
-      <c r="C21" s="21"/>
-      <c r="D21" s="21"/>
-      <c r="E21" s="24"/>
-      <c r="F21" s="21"/>
-      <c r="G21" s="21"/>
+    </row>
+    <row r="21" spans="1:8">
+      <c r="A21" s="22"/>
+      <c r="B21" s="22"/>
+      <c r="C21" s="22"/>
+      <c r="D21" s="22"/>
+      <c r="E21" s="25"/>
+      <c r="F21" s="22"/>
+      <c r="G21" s="7"/>
       <c r="H21" s="7"/>
-      <c r="I21" s="7"/>
-    </row>
-    <row r="22" spans="1:9">
-      <c r="A22" s="21"/>
-      <c r="B22" s="21"/>
-      <c r="C22" s="21"/>
-      <c r="D22" s="21"/>
-      <c r="E22" s="25"/>
-      <c r="F22" s="21"/>
-      <c r="G22" s="21"/>
+    </row>
+    <row r="22" spans="1:8">
+      <c r="A22" s="22"/>
+      <c r="B22" s="22"/>
+      <c r="C22" s="22"/>
+      <c r="D22" s="22"/>
+      <c r="E22" s="26"/>
+      <c r="F22" s="22"/>
+      <c r="G22" s="7"/>
       <c r="H22" s="7"/>
-      <c r="I22" s="7"/>
     </row>
   </sheetData>
-  <mergeCells count="29">
-    <mergeCell ref="A1:G1"/>
+  <mergeCells count="25">
+    <mergeCell ref="A1:F1"/>
     <mergeCell ref="A3:A7"/>
     <mergeCell ref="A8:A12"/>
     <mergeCell ref="A13:A17"/>
@@ -2076,10 +2044,6 @@
     <mergeCell ref="F8:F12"/>
     <mergeCell ref="F13:F17"/>
     <mergeCell ref="F18:F22"/>
-    <mergeCell ref="G3:G7"/>
-    <mergeCell ref="G8:G12"/>
-    <mergeCell ref="G13:G17"/>
-    <mergeCell ref="G18:G22"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E3:E22">
@@ -2107,7 +2071,7 @@
   <sheetData>
     <row r="1" ht="20" customHeight="1" spans="1:5">
       <c r="A1" s="15" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B1" s="15"/>
       <c r="C1" s="15"/>
@@ -2119,30 +2083,30 @@
         <v>20</v>
       </c>
       <c r="B2" s="16" t="s">
+        <v>36</v>
+      </c>
+      <c r="C2" s="16" t="s">
         <v>37</v>
       </c>
-      <c r="C2" s="16" t="s">
+      <c r="D2" s="16" t="s">
         <v>38</v>
       </c>
-      <c r="D2" s="16" t="s">
+      <c r="E2" s="16" t="s">
         <v>39</v>
-      </c>
-      <c r="E2" s="16" t="s">
-        <v>40</v>
       </c>
     </row>
     <row r="3" ht="20" customHeight="1" spans="1:5">
       <c r="A3" s="9" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B3" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="C3" s="9" t="s">
         <v>41</v>
       </c>
-      <c r="C3" s="9" t="s">
+      <c r="D3" s="17" t="s">
         <v>42</v>
-      </c>
-      <c r="D3" s="17" t="s">
-        <v>43</v>
       </c>
       <c r="E3" s="9">
         <v>1</v>
@@ -2150,16 +2114,16 @@
     </row>
     <row r="4" ht="20" customHeight="1" spans="1:5">
       <c r="A4" s="9" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B4" s="9" t="s">
+        <v>43</v>
+      </c>
+      <c r="C4" s="9" t="s">
         <v>44</v>
       </c>
-      <c r="C4" s="9" t="s">
-        <v>45</v>
-      </c>
       <c r="D4" s="17" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E4" s="9">
         <v>2</v>
@@ -2225,7 +2189,7 @@
   <sheetData>
     <row r="1" ht="22.8" spans="1:14">
       <c r="A1" s="10" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B1" s="11"/>
       <c r="C1" s="11"/>
@@ -2246,84 +2210,84 @@
         <v>20</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C2" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="D2" s="5" t="s">
         <v>47</v>
       </c>
-      <c r="D2" s="5" t="s">
+      <c r="E2" s="5" t="s">
         <v>48</v>
       </c>
-      <c r="E2" s="5" t="s">
+      <c r="F2" s="5" t="s">
         <v>49</v>
       </c>
-      <c r="F2" s="5" t="s">
+      <c r="G2" s="5" t="s">
         <v>50</v>
       </c>
-      <c r="G2" s="5" t="s">
+      <c r="H2" s="5" t="s">
         <v>51</v>
       </c>
-      <c r="H2" s="5" t="s">
+      <c r="I2" s="5" t="s">
         <v>52</v>
       </c>
-      <c r="I2" s="5" t="s">
+      <c r="J2" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="J2" s="5" t="s">
+      <c r="K2" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="K2" s="5" t="s">
+      <c r="L2" s="5" t="s">
         <v>55</v>
       </c>
-      <c r="L2" s="5" t="s">
+      <c r="M2" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="M2" s="5" t="s">
+      <c r="N2" s="5" t="s">
         <v>57</v>
-      </c>
-      <c r="N2" s="5" t="s">
-        <v>58</v>
       </c>
     </row>
     <row r="3" ht="20" customHeight="1" spans="1:14">
       <c r="A3" s="12" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B3" s="12" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C3" s="12" t="s">
+        <v>58</v>
+      </c>
+      <c r="D3" s="12" t="s">
         <v>59</v>
-      </c>
-      <c r="D3" s="12" t="s">
-        <v>60</v>
       </c>
       <c r="E3" s="12">
         <v>1</v>
       </c>
       <c r="F3" s="12" t="s">
+        <v>60</v>
+      </c>
+      <c r="G3" s="12" t="s">
         <v>61</v>
       </c>
-      <c r="G3" s="12" t="s">
+      <c r="H3" s="12" t="s">
         <v>62</v>
       </c>
-      <c r="H3" s="12" t="s">
+      <c r="I3" s="12" t="s">
+        <v>62</v>
+      </c>
+      <c r="J3" s="12" t="s">
+        <v>62</v>
+      </c>
+      <c r="K3" s="12" t="s">
+        <v>62</v>
+      </c>
+      <c r="L3" s="12" t="s">
+        <v>62</v>
+      </c>
+      <c r="M3" s="12" t="s">
         <v>63</v>
-      </c>
-      <c r="I3" s="12" t="s">
-        <v>63</v>
-      </c>
-      <c r="J3" s="12" t="s">
-        <v>63</v>
-      </c>
-      <c r="K3" s="12" t="s">
-        <v>63</v>
-      </c>
-      <c r="L3" s="12" t="s">
-        <v>63</v>
-      </c>
-      <c r="M3" s="12" t="s">
-        <v>64</v>
       </c>
       <c r="N3" s="12">
         <v>10</v>
@@ -2331,34 +2295,34 @@
     </row>
     <row r="4" ht="20" customHeight="1" spans="1:14">
       <c r="A4" s="12" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B4" s="12" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C4" s="12" t="s">
+        <v>64</v>
+      </c>
+      <c r="D4" s="12" t="s">
         <v>65</v>
-      </c>
-      <c r="D4" s="12" t="s">
-        <v>66</v>
       </c>
       <c r="E4" s="12">
         <v>2</v>
       </c>
       <c r="F4" s="12" t="s">
+        <v>66</v>
+      </c>
+      <c r="G4" s="12" t="s">
+        <v>62</v>
+      </c>
+      <c r="H4" s="12" t="s">
+        <v>62</v>
+      </c>
+      <c r="I4" s="12" t="s">
         <v>67</v>
       </c>
-      <c r="G4" s="12" t="s">
-        <v>63</v>
-      </c>
-      <c r="H4" s="12" t="s">
-        <v>63</v>
-      </c>
-      <c r="I4" s="12" t="s">
+      <c r="J4" s="12" t="s">
         <v>68</v>
-      </c>
-      <c r="J4" s="12" t="s">
-        <v>69</v>
       </c>
       <c r="K4" s="12">
         <v>360</v>
@@ -2367,7 +2331,7 @@
         <v>104857600</v>
       </c>
       <c r="M4" s="12" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="N4" s="12">
         <v>15</v>
@@ -2375,43 +2339,43 @@
     </row>
     <row r="5" ht="20" customHeight="1" spans="1:14">
       <c r="A5" s="12" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B5" s="12" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C5" s="12" t="s">
+        <v>70</v>
+      </c>
+      <c r="D5" s="12" t="s">
         <v>71</v>
-      </c>
-      <c r="D5" s="12" t="s">
-        <v>72</v>
       </c>
       <c r="E5" s="12">
         <v>1</v>
       </c>
       <c r="F5" s="12" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="G5" s="12" t="s">
+        <v>72</v>
+      </c>
+      <c r="H5" s="12" t="s">
+        <v>62</v>
+      </c>
+      <c r="I5" s="12" t="s">
+        <v>62</v>
+      </c>
+      <c r="J5" s="12" t="s">
+        <v>62</v>
+      </c>
+      <c r="K5" s="12" t="s">
+        <v>62</v>
+      </c>
+      <c r="L5" s="12" t="s">
+        <v>62</v>
+      </c>
+      <c r="M5" s="12" t="s">
         <v>73</v>
-      </c>
-      <c r="H5" s="12" t="s">
-        <v>63</v>
-      </c>
-      <c r="I5" s="12" t="s">
-        <v>63</v>
-      </c>
-      <c r="J5" s="12" t="s">
-        <v>63</v>
-      </c>
-      <c r="K5" s="12" t="s">
-        <v>63</v>
-      </c>
-      <c r="L5" s="12" t="s">
-        <v>63</v>
-      </c>
-      <c r="M5" s="12" t="s">
-        <v>74</v>
       </c>
       <c r="N5" s="12">
         <v>20</v>
@@ -2627,7 +2591,7 @@
     <row r="1" ht="23.4" spans="4:16">
       <c r="D1" s="4"/>
       <c r="E1" s="4" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="F1" s="4"/>
       <c r="G1" s="4"/>
@@ -2646,43 +2610,43 @@
         <v>20</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="D2" s="6" t="s">
+        <v>75</v>
+      </c>
+      <c r="E2" s="6" t="s">
         <v>76</v>
       </c>
-      <c r="E2" s="6" t="s">
+      <c r="F2" s="6" t="s">
         <v>77</v>
       </c>
-      <c r="F2" s="6" t="s">
+      <c r="G2" s="6" t="s">
         <v>78</v>
       </c>
-      <c r="G2" s="6" t="s">
+      <c r="H2" s="6" t="s">
         <v>79</v>
       </c>
-      <c r="H2" s="6" t="s">
+      <c r="I2" s="6" t="s">
         <v>80</v>
       </c>
-      <c r="I2" s="6" t="s">
+      <c r="J2" s="6" t="s">
         <v>81</v>
       </c>
-      <c r="J2" s="6" t="s">
+      <c r="K2" s="6" t="s">
         <v>82</v>
       </c>
-      <c r="K2" s="6" t="s">
+      <c r="L2" s="6" t="s">
         <v>83</v>
       </c>
-      <c r="L2" s="6" t="s">
+      <c r="M2" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="N2" s="6" t="s">
         <v>84</v>
-      </c>
-      <c r="M2" s="6" t="s">
-        <v>49</v>
-      </c>
-      <c r="N2" s="6" t="s">
-        <v>85</v>
       </c>
       <c r="O2" s="6" t="s">
         <v>24</v>
@@ -2738,7 +2702,7 @@
   <sheetData>
     <row r="1" s="1" customFormat="1" ht="30" customHeight="1" spans="1:2">
       <c r="A1" s="2" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>22</v>
@@ -2749,47 +2713,47 @@
         <v>20</v>
       </c>
       <c r="B2" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="3" ht="20" customHeight="1" spans="1:2">
       <c r="A3" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B3" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="4" ht="20" customHeight="1" spans="1:2">
       <c r="A4" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B4" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="5" ht="20" customHeight="1" spans="1:2">
       <c r="A5" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B5" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1" spans="1:2">
       <c r="A6" t="s">
+        <v>90</v>
+      </c>
+      <c r="B6" t="s">
         <v>91</v>
-      </c>
-      <c r="B6" t="s">
-        <v>92</v>
       </c>
     </row>
     <row r="7" ht="20" customHeight="1" spans="1:2">
       <c r="A7" t="s">
+        <v>92</v>
+      </c>
+      <c r="B7" t="s">
         <v>93</v>
-      </c>
-      <c r="B7" t="s">
-        <v>94</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: implement trainer dashboard backend services and frontend file upload utilities
</commit_message>
<xml_diff>
--- a/doc/templates/Hango_Course_Import_Template.xlsx
+++ b/doc/templates/Hango_Course_Import_Template.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="14100" windowHeight="9000" firstSheet="2" activeTab="2"/>
+    <workbookView windowWidth="15084" windowHeight="6072" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="README_AND_RULES" sheetId="1" r:id="rId1"/>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="118" uniqueCount="109">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="117" uniqueCount="108">
   <si>
     <t>Hango Course Import Template - Rules</t>
   </si>
@@ -651,9 +651,6 @@
   </si>
   <si>
     <t>Lesson 1: Vid</t>
-  </si>
-  <si>
-    <t>https://www.youtube.com/watch?v=MpiWuR-yL9k</t>
   </si>
   <si>
     <t>Text</t>
@@ -2890,12 +2887,8 @@
       <c r="C8" s="18" t="s">
         <v>82</v>
       </c>
-      <c r="D8" s="21" t="s">
-        <v>83</v>
-      </c>
-      <c r="E8" s="19">
-        <v>15</v>
-      </c>
+      <c r="D8" s="21"/>
+      <c r="E8" s="19"/>
       <c r="F8" s="19"/>
       <c r="G8" s="20"/>
       <c r="H8" s="20"/>
@@ -2921,10 +2914,10 @@
         <v>3</v>
       </c>
       <c r="B10" s="18" t="s">
+        <v>83</v>
+      </c>
+      <c r="C10" s="18" t="s">
         <v>84</v>
-      </c>
-      <c r="C10" s="18" t="s">
-        <v>85</v>
       </c>
       <c r="D10" s="18"/>
       <c r="E10" s="19">
@@ -2997,7 +2990,7 @@
         <v>79</v>
       </c>
       <c r="C15" s="18" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D15" s="18"/>
       <c r="E15" s="19"/>
@@ -3026,10 +3019,10 @@
         <v>5</v>
       </c>
       <c r="B17" s="18" t="s">
+        <v>86</v>
+      </c>
+      <c r="C17" s="18" t="s">
         <v>87</v>
-      </c>
-      <c r="C17" s="18" t="s">
-        <v>88</v>
       </c>
       <c r="D17" s="18"/>
       <c r="E17" s="22">
@@ -3132,9 +3125,6 @@
       <formula1>"BEGINNER,INTERMEDIATE,ADVANCE"</formula1>
     </dataValidation>
   </dataValidations>
-  <hyperlinks>
-    <hyperlink ref="D8" r:id="rId1" display="https://www.youtube.com/watch?v=MpiWuR-yL9k" tooltip="https://www.youtube.com/watch?v=MpiWuR-yL9k"/>
-  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>
 </worksheet>
@@ -3159,7 +3149,7 @@
     <row r="1" ht="23.4" spans="5:17">
       <c r="E1" s="2"/>
       <c r="F1" s="2" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="G1" s="2"/>
       <c r="H1" s="2"/>
@@ -3175,40 +3165,40 @@
     </row>
     <row r="2" s="1" customFormat="1" ht="30" customHeight="1" spans="1:14">
       <c r="A2" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="B2" s="3" t="s">
         <v>90</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="C2" s="3" t="s">
         <v>91</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="D2" s="3" t="s">
         <v>92</v>
       </c>
-      <c r="D2" s="3" t="s">
+      <c r="E2" s="3" t="s">
         <v>93</v>
       </c>
-      <c r="E2" s="3" t="s">
+      <c r="F2" s="3" t="s">
         <v>94</v>
       </c>
-      <c r="F2" s="3" t="s">
+      <c r="G2" s="3" t="s">
         <v>95</v>
       </c>
-      <c r="G2" s="3" t="s">
+      <c r="H2" s="3" t="s">
         <v>96</v>
       </c>
-      <c r="H2" s="3" t="s">
+      <c r="I2" s="3" t="s">
         <v>97</v>
       </c>
-      <c r="I2" s="3" t="s">
+      <c r="J2" s="3" t="s">
         <v>98</v>
       </c>
-      <c r="J2" s="3" t="s">
+      <c r="K2" s="3" t="s">
         <v>99</v>
       </c>
-      <c r="K2" s="3" t="s">
+      <c r="L2" s="3" t="s">
         <v>100</v>
-      </c>
-      <c r="L2" s="3" t="s">
-        <v>101</v>
       </c>
       <c r="M2" s="3" t="s">
         <v>66</v>
@@ -3219,32 +3209,32 @@
     </row>
     <row r="3" ht="47" customHeight="1" spans="1:17">
       <c r="A3" s="4" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="C3" s="5"/>
       <c r="D3" s="5" t="s">
+        <v>102</v>
+      </c>
+      <c r="E3" s="5" t="s">
         <v>103</v>
       </c>
-      <c r="E3" s="5" t="s">
+      <c r="F3" s="6" t="s">
         <v>104</v>
       </c>
-      <c r="F3" s="6" t="s">
+      <c r="G3" s="6" t="s">
         <v>105</v>
       </c>
-      <c r="G3" s="6" t="s">
+      <c r="H3" s="6" t="s">
         <v>106</v>
       </c>
-      <c r="H3" s="6" t="s">
+      <c r="I3" s="6" t="s">
+        <v>103</v>
+      </c>
+      <c r="J3" s="6" t="s">
         <v>107</v>
-      </c>
-      <c r="I3" s="6" t="s">
-        <v>104</v>
-      </c>
-      <c r="J3" s="6" t="s">
-        <v>108</v>
       </c>
       <c r="K3" s="6"/>
       <c r="L3" s="6"/>

</xml_diff>